<commit_message>
Add quest engine foundation: GameStats, QuestDef, QuestManager
</commit_message>
<xml_diff>
--- a/docs/documentation/plants.xlsx
+++ b/docs/documentation/plants.xlsx
@@ -1,21 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\m1382\Desktop\CTR\ta\ap\project-documents\assets\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/amirali/Desktop/ApProject/advanced-programming-sut-2026/docs/documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4D95D140-95DA-40E6-A2CE-D8502E580581}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{279333FE-5F86-7645-ACA7-73BAA76445FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="25600" windowHeight="14700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plants" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -989,7 +1002,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -1000,6 +1013,13 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -1029,7 +1049,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1055,27 +1075,14 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" readingOrder="2"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="4">
-    <dxf>
-      <border>
-        <left style="thin">
-          <color rgb="FF356854"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF356854"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF356854"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF356854"/>
-        </bottom>
-      </border>
-    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1100,13 +1107,29 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF356854"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF356854"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF356854"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF356854"/>
+        </bottom>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="1">
     <tableStyle name="Plants-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="0"/>
-      <tableStyleElement type="headerRow" dxfId="3"/>
-      <tableStyleElement type="firstRowStripe" dxfId="2"/>
-      <tableStyleElement type="secondRowStripe" dxfId="1"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="3"/>
+      <tableStyleElement type="headerRow" dxfId="2"/>
+      <tableStyleElement type="firstRowStripe" dxfId="1"/>
+      <tableStyleElement type="secondRowStripe" dxfId="0"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -1349,24 +1372,24 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:N70"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="10.26953125" customWidth="1"/>
-    <col min="2" max="2" width="16.453125" customWidth="1"/>
-    <col min="3" max="3" width="16.26953125" customWidth="1"/>
-    <col min="4" max="4" width="20.6328125" customWidth="1"/>
-    <col min="5" max="5" width="12.26953125" customWidth="1"/>
-    <col min="6" max="6" width="15.08984375" customWidth="1"/>
-    <col min="7" max="7" width="15.26953125" customWidth="1"/>
-    <col min="8" max="8" width="73.90625" customWidth="1"/>
+    <col min="1" max="1" width="10.33203125" customWidth="1"/>
+    <col min="2" max="2" width="16.5" customWidth="1"/>
+    <col min="3" max="3" width="16.33203125" customWidth="1"/>
+    <col min="4" max="4" width="20.6640625" customWidth="1"/>
+    <col min="5" max="5" width="12.33203125" customWidth="1"/>
+    <col min="6" max="6" width="15.1640625" customWidth="1"/>
+    <col min="7" max="7" width="15.33203125" customWidth="1"/>
+    <col min="8" max="8" width="73.83203125" customWidth="1"/>
     <col min="9" max="9" width="38" customWidth="1"/>
-    <col min="10" max="10" width="14.453125" customWidth="1"/>
-    <col min="11" max="11" width="19.7265625" customWidth="1"/>
-    <col min="12" max="12" width="19.90625" customWidth="1"/>
-    <col min="13" max="14" width="21.90625" customWidth="1"/>
+    <col min="10" max="10" width="14.5" customWidth="1"/>
+    <col min="11" max="11" width="19.6640625" customWidth="1"/>
+    <col min="12" max="12" width="19.83203125" customWidth="1"/>
+    <col min="13" max="14" width="21.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1403,14 +1426,14 @@
       <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="9" t="s">
         <v>12</v>
       </c>
       <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -1454,7 +1477,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -1498,7 +1521,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -1542,7 +1565,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -1586,7 +1609,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -1630,7 +1653,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -1674,7 +1697,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -1718,7 +1741,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -1762,7 +1785,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -1806,7 +1829,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -1850,7 +1873,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="5">
         <v>11</v>
       </c>
@@ -1894,7 +1917,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -1938,7 +1961,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="14" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -1982,7 +2005,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="15" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="5">
         <v>14</v>
       </c>
@@ -2026,7 +2049,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="16" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="5">
         <v>15</v>
       </c>
@@ -2070,7 +2093,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="17" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -2114,7 +2137,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="18" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -2158,7 +2181,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="19" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -2202,7 +2225,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="5">
         <v>19</v>
       </c>
@@ -2246,7 +2269,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="21" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A21" s="5">
         <v>20</v>
       </c>
@@ -2290,7 +2313,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="22" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -2334,7 +2357,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="23" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="2">
         <v>22</v>
       </c>
@@ -2378,7 +2401,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="24" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="2">
         <v>23</v>
       </c>
@@ -2422,7 +2445,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="25" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="2">
         <v>24</v>
       </c>
@@ -2466,7 +2489,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="26" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="2">
         <v>25</v>
       </c>
@@ -2510,7 +2533,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="27" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="2">
         <v>26</v>
       </c>
@@ -2554,7 +2577,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="28" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="2">
         <v>27</v>
       </c>
@@ -2598,7 +2621,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="29" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A29" s="2">
         <v>28</v>
       </c>
@@ -2642,7 +2665,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="30" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A30" s="2">
         <v>29</v>
       </c>
@@ -2686,7 +2709,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="31" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A31" s="2">
         <v>30</v>
       </c>
@@ -2730,7 +2753,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="32" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A32" s="2">
         <v>31</v>
       </c>
@@ -2774,7 +2797,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="33" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A33" s="2">
         <v>32</v>
       </c>
@@ -2818,7 +2841,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="34" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A34" s="2">
         <v>33</v>
       </c>
@@ -2862,7 +2885,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="35" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A35" s="5">
         <v>34</v>
       </c>
@@ -2906,7 +2929,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="36" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A36" s="2">
         <v>35</v>
       </c>
@@ -2950,7 +2973,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="37" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A37" s="2">
         <v>36</v>
       </c>
@@ -2994,7 +3017,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="38" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A38" s="2">
         <v>37</v>
       </c>
@@ -3038,7 +3061,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="39" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A39" s="2">
         <v>38</v>
       </c>
@@ -3082,7 +3105,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="40" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A40" s="2">
         <v>39</v>
       </c>
@@ -3126,7 +3149,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="41" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A41" s="2">
         <v>40</v>
       </c>
@@ -3170,7 +3193,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="42" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A42" s="5">
         <v>41</v>
       </c>
@@ -3214,7 +3237,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="43" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A43" s="5">
         <v>42</v>
       </c>
@@ -3258,7 +3281,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="44" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A44" s="5">
         <v>43</v>
       </c>
@@ -3302,7 +3325,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="45" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A45" s="2">
         <v>44</v>
       </c>
@@ -3346,7 +3369,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="46" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A46" s="2">
         <v>45</v>
       </c>
@@ -3390,7 +3413,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="47" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A47" s="2">
         <v>46</v>
       </c>
@@ -3434,7 +3457,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="48" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A48" s="2">
         <v>47</v>
       </c>
@@ -3478,7 +3501,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="49" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A49" s="5">
         <v>48</v>
       </c>
@@ -3522,7 +3545,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="50" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A50" s="2">
         <v>49</v>
       </c>
@@ -3566,7 +3589,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="51" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A51" s="2">
         <v>50</v>
       </c>
@@ -3610,7 +3633,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="52" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A52" s="2">
         <v>51</v>
       </c>
@@ -3654,7 +3677,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="53" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A53" s="2">
         <v>52</v>
       </c>
@@ -3698,7 +3721,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="54" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A54" s="2">
         <v>53</v>
       </c>
@@ -3742,7 +3765,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="55" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A55" s="5">
         <v>54</v>
       </c>
@@ -3786,7 +3809,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="56" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A56" s="5">
         <v>55</v>
       </c>
@@ -3830,7 +3853,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="57" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A57" s="2">
         <v>56</v>
       </c>
@@ -3874,7 +3897,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A58" s="2">
         <v>57</v>
       </c>
@@ -3918,7 +3941,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="59" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A59" s="2">
         <v>58</v>
       </c>
@@ -3962,7 +3985,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="60" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A60" s="2">
         <v>59</v>
       </c>
@@ -4006,7 +4029,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="61" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A61" s="2">
         <v>60</v>
       </c>
@@ -4050,7 +4073,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="62" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A62" s="2">
         <v>61</v>
       </c>
@@ -4094,7 +4117,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="63" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A63" s="2">
         <v>62</v>
       </c>
@@ -4138,7 +4161,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="64" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A64" s="2">
         <v>63</v>
       </c>
@@ -4182,7 +4205,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="65" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A65" s="2">
         <v>64</v>
       </c>
@@ -4226,7 +4249,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="66" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A66" s="2">
         <v>65</v>
       </c>
@@ -4270,7 +4293,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="67" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A67" s="2">
         <v>66</v>
       </c>
@@ -4314,7 +4337,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="68" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A68" s="2">
         <v>67</v>
       </c>
@@ -4358,7 +4381,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="69" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A69" s="2">
         <v>68</v>
       </c>
@@ -4402,7 +4425,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="70" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A70" s="2">
         <v>69</v>
       </c>

</xml_diff>